<commit_message>
Update attendance sheet for Introduction to Programming 2026-27
</commit_message>
<xml_diff>
--- a/Folha_de_Presencas_Introducao_a_Programacao_2026-27.xlsx
+++ b/Folha_de_Presencas_Introducao_a_Programacao_2026-27.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18600" windowHeight="6350"/>
+    <workbookView windowWidth="19200" windowHeight="6800"/>
   </bookViews>
   <sheets>
     <sheet name="Presenças" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="58">
   <si>
     <t>REGISTO DE PRESENÇAS</t>
   </si>
@@ -2342,8 +2342,12 @@
       </c>
       <c r="E9" s="19"/>
       <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="19"/>
+      <c r="G9" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="H9" s="19" t="s">
+        <v>19</v>
+      </c>
       <c r="I9" s="19"/>
       <c r="J9" s="19"/>
       <c r="K9" s="19"/>
@@ -2399,9 +2403,15 @@
       <c r="F10" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G10" s="27"/>
-      <c r="H10" s="27"/>
-      <c r="I10" s="27"/>
+      <c r="G10" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="H10" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="I10" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="J10" s="27"/>
       <c r="K10" s="27"/>
       <c r="L10" s="27"/>
@@ -2452,9 +2462,15 @@
       </c>
       <c r="E11" s="27"/>
       <c r="F11" s="27"/>
-      <c r="G11" s="27"/>
-      <c r="H11" s="27"/>
-      <c r="I11" s="27"/>
+      <c r="G11" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="H11" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="I11" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="J11" s="27"/>
       <c r="K11" s="27"/>
       <c r="L11" s="27"/>
@@ -2509,9 +2525,15 @@
       <c r="F12" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G12" s="27"/>
-      <c r="H12" s="27"/>
-      <c r="I12" s="27"/>
+      <c r="G12" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="H12" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="I12" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="J12" s="27"/>
       <c r="K12" s="27"/>
       <c r="L12" s="27"/>
@@ -2562,8 +2584,12 @@
       </c>
       <c r="E13" s="27"/>
       <c r="F13" s="27"/>
-      <c r="G13" s="27"/>
-      <c r="H13" s="27"/>
+      <c r="G13" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="H13" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="I13" s="27"/>
       <c r="J13" s="27"/>
       <c r="K13" s="27"/>
@@ -2615,8 +2641,12 @@
       </c>
       <c r="E14" s="27"/>
       <c r="F14" s="27"/>
-      <c r="G14" s="27"/>
-      <c r="H14" s="27"/>
+      <c r="G14" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="H14" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="I14" s="27"/>
       <c r="J14" s="27"/>
       <c r="K14" s="27"/>
@@ -2672,9 +2702,15 @@
       <c r="F15" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G15" s="27"/>
-      <c r="H15" s="27"/>
-      <c r="I15" s="27"/>
+      <c r="G15" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="H15" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="I15" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="J15" s="27"/>
       <c r="K15" s="27"/>
       <c r="L15" s="27"/>
@@ -2729,9 +2765,15 @@
       <c r="F16" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G16" s="27"/>
-      <c r="H16" s="27"/>
-      <c r="I16" s="27"/>
+      <c r="G16" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="H16" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="I16" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="J16" s="27"/>
       <c r="K16" s="27"/>
       <c r="L16" s="27"/>
@@ -2786,9 +2828,15 @@
       <c r="F17" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G17" s="27"/>
-      <c r="H17" s="27"/>
-      <c r="I17" s="27"/>
+      <c r="G17" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="H17" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="I17" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="J17" s="27"/>
       <c r="K17" s="27"/>
       <c r="L17" s="27"/>
@@ -2843,9 +2891,15 @@
       <c r="F18" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G18" s="27"/>
-      <c r="H18" s="27"/>
-      <c r="I18" s="27"/>
+      <c r="G18" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="H18" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="I18" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="J18" s="27"/>
       <c r="K18" s="27"/>
       <c r="L18" s="27"/>
@@ -2896,8 +2950,12 @@
       </c>
       <c r="E19" s="27"/>
       <c r="F19" s="27"/>
-      <c r="G19" s="27"/>
-      <c r="H19" s="27"/>
+      <c r="G19" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="H19" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="I19" s="27"/>
       <c r="J19" s="27"/>
       <c r="K19" s="27"/>
@@ -2953,8 +3011,12 @@
       <c r="F20" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G20" s="27"/>
-      <c r="H20" s="27"/>
+      <c r="G20" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="H20" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="I20" s="27"/>
       <c r="J20" s="27"/>
       <c r="K20" s="27"/>
@@ -3010,9 +3072,15 @@
       <c r="F21" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G21" s="27"/>
-      <c r="H21" s="27"/>
-      <c r="I21" s="27"/>
+      <c r="G21" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="H21" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="I21" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="J21" s="27"/>
       <c r="K21" s="27"/>
       <c r="L21" s="27"/>
@@ -3067,9 +3135,15 @@
       <c r="F22" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G22" s="27"/>
-      <c r="H22" s="27"/>
-      <c r="I22" s="27"/>
+      <c r="G22" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="H22" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="I22" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="J22" s="27"/>
       <c r="K22" s="27"/>
       <c r="L22" s="27"/>
@@ -3122,8 +3196,12 @@
         <v>19</v>
       </c>
       <c r="F23" s="27"/>
-      <c r="G23" s="27"/>
-      <c r="H23" s="27"/>
+      <c r="G23" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="H23" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="I23" s="27"/>
       <c r="J23" s="27"/>
       <c r="K23" s="27"/>
@@ -3179,9 +3257,15 @@
       <c r="F24" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G24" s="27"/>
-      <c r="H24" s="27"/>
-      <c r="I24" s="27"/>
+      <c r="G24" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="H24" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="I24" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="J24" s="27"/>
       <c r="K24" s="27"/>
       <c r="L24" s="27"/>
@@ -3236,9 +3320,15 @@
       <c r="F25" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G25" s="27"/>
-      <c r="H25" s="27"/>
-      <c r="I25" s="27"/>
+      <c r="G25" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="H25" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="I25" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="J25" s="27"/>
       <c r="K25" s="27"/>
       <c r="L25" s="27"/>
@@ -3293,9 +3383,15 @@
       <c r="F26" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="G26" s="36"/>
-      <c r="H26" s="36"/>
-      <c r="I26" s="36"/>
+      <c r="G26" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="H26" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="I26" s="36" t="s">
+        <v>19</v>
+      </c>
       <c r="J26" s="36"/>
       <c r="K26" s="36"/>
       <c r="L26" s="36"/>
@@ -3390,15 +3486,15 @@
       </c>
       <c r="G28" s="42">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="H28" s="42">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="I28" s="42">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J28" s="42">
         <f t="shared" si="3"/>
@@ -3736,7 +3832,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="C9:AE26">
+    <dataValidation type="list" sqref="G9:G26 H11:H26 C9:F10 H9:AE10 C11:F26 I11:AE26">
       <formula1>"P,F,J"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Update attendance sheet for Introduction to Programming 2026-27 and remove outdated file
</commit_message>
<xml_diff>
--- a/Folha_de_Presencas_Introducao_a_Programacao_2026-27.xlsx
+++ b/Folha_de_Presencas_Introducao_a_Programacao_2026-27.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="58">
   <si>
     <t>REGISTO DE PRESENÇAS</t>
   </si>
@@ -1435,11 +1435,11 @@
     <dxf>
       <font>
         <b val="1"/>
-        <color rgb="FF14583B"/>
+        <color rgb="FF285785"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFDCF2E8"/>
+          <bgColor rgb="FFDEEDFA"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1457,11 +1457,11 @@
     <dxf>
       <font>
         <b val="1"/>
-        <color rgb="FF285785"/>
+        <color rgb="FF14583B"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFDEEDFA"/>
+          <bgColor rgb="FFDCF2E8"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2345,9 +2345,7 @@
       <c r="G9" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="H9" s="19" t="s">
-        <v>19</v>
-      </c>
+      <c r="H9" s="19"/>
       <c r="I9" s="19"/>
       <c r="J9" s="19"/>
       <c r="K9" s="19"/>
@@ -2462,12 +2460,10 @@
       </c>
       <c r="E11" s="27"/>
       <c r="F11" s="27"/>
-      <c r="G11" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="H11" s="27" t="s">
-        <v>19</v>
-      </c>
+      <c r="G11" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="H11" s="27"/>
       <c r="I11" s="27" t="s">
         <v>19</v>
       </c>
@@ -2584,12 +2580,8 @@
       </c>
       <c r="E13" s="27"/>
       <c r="F13" s="27"/>
-      <c r="G13" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="H13" s="27" t="s">
-        <v>19</v>
-      </c>
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
       <c r="I13" s="27"/>
       <c r="J13" s="27"/>
       <c r="K13" s="27"/>
@@ -2641,12 +2633,8 @@
       </c>
       <c r="E14" s="27"/>
       <c r="F14" s="27"/>
-      <c r="G14" s="27" t="s">
-        <v>19</v>
-      </c>
-      <c r="H14" s="27" t="s">
-        <v>19</v>
-      </c>
+      <c r="G14" s="27"/>
+      <c r="H14" s="27"/>
       <c r="I14" s="27"/>
       <c r="J14" s="27"/>
       <c r="K14" s="27"/>
@@ -2702,7 +2690,7 @@
       <c r="F15" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G15" s="19" t="s">
+      <c r="G15" s="27" t="s">
         <v>19</v>
       </c>
       <c r="H15" s="27" t="s">
@@ -2828,7 +2816,7 @@
       <c r="F17" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G17" s="19" t="s">
+      <c r="G17" s="27" t="s">
         <v>19</v>
       </c>
       <c r="H17" s="27" t="s">
@@ -2950,12 +2938,8 @@
       </c>
       <c r="E19" s="27"/>
       <c r="F19" s="27"/>
-      <c r="G19" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="H19" s="27" t="s">
-        <v>19</v>
-      </c>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
       <c r="I19" s="27"/>
       <c r="J19" s="27"/>
       <c r="K19" s="27"/>
@@ -3014,9 +2998,7 @@
       <c r="G20" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="H20" s="27" t="s">
-        <v>19</v>
-      </c>
+      <c r="H20" s="27"/>
       <c r="I20" s="27"/>
       <c r="J20" s="27"/>
       <c r="K20" s="27"/>
@@ -3072,7 +3054,7 @@
       <c r="F21" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G21" s="19" t="s">
+      <c r="G21" s="27" t="s">
         <v>19</v>
       </c>
       <c r="H21" s="27" t="s">
@@ -3196,12 +3178,10 @@
         <v>19</v>
       </c>
       <c r="F23" s="27"/>
-      <c r="G23" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="H23" s="27" t="s">
-        <v>19</v>
-      </c>
+      <c r="G23" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="H23" s="27"/>
       <c r="I23" s="27"/>
       <c r="J23" s="27"/>
       <c r="K23" s="27"/>
@@ -3320,7 +3300,7 @@
       <c r="F25" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G25" s="19" t="s">
+      <c r="G25" s="27" t="s">
         <v>19</v>
       </c>
       <c r="H25" s="27" t="s">
@@ -3383,10 +3363,10 @@
       <c r="F26" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="G26" s="27" t="s">
-        <v>19</v>
-      </c>
-      <c r="H26" s="27" t="s">
+      <c r="G26" s="36" t="s">
+        <v>19</v>
+      </c>
+      <c r="H26" s="36" t="s">
         <v>19</v>
       </c>
       <c r="I26" s="36" t="s">
@@ -3486,11 +3466,11 @@
       </c>
       <c r="G28" s="42">
         <f t="shared" si="3"/>
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="H28" s="42">
         <f t="shared" si="3"/>
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="I28" s="42">
         <f t="shared" si="3"/>
@@ -3820,19 +3800,30 @@
       <c r="AH34" s="1"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C9:AE26">
-    <cfRule type="expression" dxfId="0" priority="1">
+  <conditionalFormatting sqref="I9:I26">
+    <cfRule type="expression" dxfId="0" priority="3">
+      <formula>I9="J"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>I9="F"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="1">
+      <formula>I9="P"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C9:H26;J9:AE26">
+    <cfRule type="expression" dxfId="2" priority="4">
       <formula>C9="P"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="1" priority="5">
       <formula>C9="F"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="0" priority="6">
       <formula>C9="J"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="G9:G26 H11:H26 C9:F10 H9:AE10 C11:F26 I11:AE26">
+    <dataValidation type="list" sqref="I9:I26 C9:H26 J9:AE26">
       <formula1>"P,F,J"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Update attendance sheet for Introduction to Programming 2026-27 and remove temporary file
</commit_message>
<xml_diff>
--- a/Folha_de_Presencas_Introducao_a_Programacao_2026-27.xlsx
+++ b/Folha_de_Presencas_Introducao_a_Programacao_2026-27.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="58">
   <si>
     <t>REGISTO DE PRESENÇAS</t>
   </si>
@@ -2350,7 +2350,9 @@
       <c r="J9" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="K9" s="19"/>
+      <c r="K9" s="19" t="s">
+        <v>19</v>
+      </c>
       <c r="L9" s="19"/>
       <c r="M9" s="19"/>
       <c r="N9" s="19"/>
@@ -2415,7 +2417,9 @@
       <c r="J10" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="K10" s="27"/>
+      <c r="K10" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="L10" s="27"/>
       <c r="M10" s="27"/>
       <c r="N10" s="27"/>
@@ -2474,7 +2478,9 @@
       <c r="J11" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="K11" s="27"/>
+      <c r="K11" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="L11" s="27"/>
       <c r="M11" s="27"/>
       <c r="N11" s="27"/>
@@ -2539,7 +2545,9 @@
       <c r="J12" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="K12" s="27"/>
+      <c r="K12" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="L12" s="27"/>
       <c r="M12" s="27"/>
       <c r="N12" s="27"/>
@@ -2710,7 +2718,9 @@
       <c r="J15" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="K15" s="27"/>
+      <c r="K15" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="L15" s="27"/>
       <c r="M15" s="27"/>
       <c r="N15" s="27"/>
@@ -2840,7 +2850,9 @@
       <c r="J17" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="K17" s="27"/>
+      <c r="K17" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="L17" s="27"/>
       <c r="M17" s="27"/>
       <c r="N17" s="27"/>
@@ -2905,7 +2917,9 @@
       <c r="J18" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="K18" s="27"/>
+      <c r="K18" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="L18" s="27"/>
       <c r="M18" s="27"/>
       <c r="N18" s="27"/>
@@ -3082,7 +3096,9 @@
       <c r="J21" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="K21" s="27"/>
+      <c r="K21" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="L21" s="27"/>
       <c r="M21" s="27"/>
       <c r="N21" s="27"/>
@@ -3147,7 +3163,9 @@
       <c r="J22" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="K22" s="27"/>
+      <c r="K22" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="L22" s="27"/>
       <c r="M22" s="27"/>
       <c r="N22" s="27"/>
@@ -3269,7 +3287,9 @@
       <c r="J24" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="K24" s="27"/>
+      <c r="K24" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="L24" s="27"/>
       <c r="M24" s="27"/>
       <c r="N24" s="27"/>
@@ -3334,7 +3354,9 @@
       <c r="J25" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="K25" s="27"/>
+      <c r="K25" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="L25" s="27"/>
       <c r="M25" s="27"/>
       <c r="N25" s="27"/>
@@ -3399,7 +3421,9 @@
       <c r="J26" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="K26" s="36"/>
+      <c r="K26" s="36" t="s">
+        <v>19</v>
+      </c>
       <c r="L26" s="36"/>
       <c r="M26" s="36"/>
       <c r="N26" s="36"/>
@@ -3508,7 +3532,7 @@
       </c>
       <c r="K28" s="42">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="L28" s="42">
         <f t="shared" si="3"/>

</xml_diff>

<commit_message>
Update attendance sheet for Introdução à Programação 2026-27
</commit_message>
<xml_diff>
--- a/Folha_de_Presencas_Introducao_a_Programacao_2026-27.xlsx
+++ b/Folha_de_Presencas_Introducao_a_Programacao_2026-27.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="58">
   <si>
     <t>REGISTO DE PRESENÇAS</t>
   </si>
@@ -2353,7 +2353,9 @@
       <c r="K9" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="L9" s="19"/>
+      <c r="L9" s="19" t="s">
+        <v>19</v>
+      </c>
       <c r="M9" s="19"/>
       <c r="N9" s="19"/>
       <c r="O9" s="19"/>
@@ -2481,7 +2483,9 @@
       <c r="K11" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="L11" s="27"/>
+      <c r="L11" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="M11" s="27"/>
       <c r="N11" s="27"/>
       <c r="O11" s="27"/>
@@ -2548,7 +2552,9 @@
       <c r="K12" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="L12" s="27"/>
+      <c r="L12" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="M12" s="27"/>
       <c r="N12" s="27"/>
       <c r="O12" s="27"/>
@@ -2721,7 +2727,9 @@
       <c r="K15" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="L15" s="27"/>
+      <c r="L15" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="M15" s="27"/>
       <c r="N15" s="27"/>
       <c r="O15" s="27"/>
@@ -2920,7 +2928,9 @@
       <c r="K18" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="L18" s="27"/>
+      <c r="L18" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="M18" s="27"/>
       <c r="N18" s="27"/>
       <c r="O18" s="27"/>
@@ -3166,7 +3176,9 @@
       <c r="K22" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="L22" s="27"/>
+      <c r="L22" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="M22" s="27"/>
       <c r="N22" s="27"/>
       <c r="O22" s="27"/>
@@ -3357,7 +3369,9 @@
       <c r="K25" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="L25" s="27"/>
+      <c r="L25" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="M25" s="27"/>
       <c r="N25" s="27"/>
       <c r="O25" s="27"/>
@@ -3536,7 +3550,7 @@
       </c>
       <c r="L28" s="42">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="M28" s="42">
         <f t="shared" si="3"/>

</xml_diff>